<commit_message>
📊 BIST Screener | 12.05.2026 17:31 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-12.xlsx
+++ b/data/bist_screener_2026-05-12.xlsx
@@ -25823,21 +25823,21 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>17.89</v>
+        <v>14.47</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0438</v>
-      </c>
-      <c r="D585" s="9" t="n">
-        <v>66660000</v>
+        <v>-0.0366</v>
+      </c>
+      <c r="D585" s="7" t="n">
+        <v>32410000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>54.49</v>
+        <v>55.48</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25845,12 +25845,12 @@
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25858,21 +25858,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>14.47</v>
+        <v>79.3</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0366</v>
-      </c>
-      <c r="D586" s="3" t="n">
-        <v>32410000</v>
+        <v>-0.021</v>
+      </c>
+      <c r="D586" s="5" t="n">
+        <v>171630</v>
       </c>
       <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>55.48</v>
+        <v>11.3</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25880,53 +25880,43 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L586" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr"/>
       <c r="M586" s="2" t="inlineStr"/>
     </row>
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>2.63</v>
+        <v>45.46</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0295</v>
+        <v>0.0102</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>28760000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>6120000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>41.18</v>
+        <v>67.47</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25934,56 +25924,48 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>30.7</v>
+        <v>80.04000000000001</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0007000000000000001</v>
+        <v>-0.009399999999999999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>26120000</v>
+        <v>10710000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>68.69</v>
+        <v>43.25</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
-      <c r="K588" s="2" t="inlineStr">
-        <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K588" s="2" t="inlineStr"/>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>79.3</v>
+        <v>2.88</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.021</v>
+        <v>-0.0368</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>171630</v>
+        <v>190570000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>11.3</v>
+        <v>52.36</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -25994,38 +25976,36 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L589" s="6" t="inlineStr"/>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>6.34</v>
+        <v>17.89</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0745</v>
+        <v>-0.0438</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>57090000</v>
-      </c>
-      <c r="E590" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>66660000</v>
+      </c>
+      <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>51.71</v>
+        <v>54.49</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J590" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I590" s="2" t="inlineStr"/>
+      <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26033,7 +26013,7 @@
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26041,60 +26021,60 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>31.36</v>
+        <v>9.6</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0058</v>
+        <v>-0.0194</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>14110000</v>
+        <v>961350</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.95</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>60.8</v>
+        <v>60.81</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>6.06</v>
+        <v>31.36</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.008199999999999999</v>
+        <v>0.0058</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>44330000</v>
+        <v>14110000</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.8667</v>
+        <v>0.2667</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>67.06999999999999</v>
+        <v>60.8</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26102,12 +26082,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26185,34 +26165,40 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>45.46</v>
+        <v>19.78</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0102</v>
+        <v>-0.0639</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>6120000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>711640</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>67.47</v>
+        <v>60.87</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26220,137 +26206,163 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>35.76</v>
+        <v>76.8</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0245</v>
+        <v>-0.0235</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>5260000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>60180</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>59.16</v>
+        <v>43.15</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>TCELL</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>244.25</v>
+        <v>115</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0338</v>
+        <v>-0.0566</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>10010</v>
+        <v>21130000</v>
       </c>
       <c r="E597" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.4894</v>
       </c>
       <c r="F597" s="7" t="n">
-        <v>45.91</v>
-      </c>
-      <c r="G597" s="6" t="inlineStr"/>
+        <v>50.2</v>
+      </c>
+      <c r="G597" s="7" t="n">
+        <v>13.6</v>
+      </c>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>0.0735</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>0.1091</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>İletişim</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST İLETİŞİM, BIST HİZMETLER, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>6.12</v>
+        <v>35.16</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.006500000000000001</v>
+        <v>-0.0228</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>7340000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>5700000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>53.81</v>
-      </c>
-      <c r="G598" s="2" t="inlineStr"/>
+        <v>42.83</v>
+      </c>
+      <c r="G598" s="3" t="n">
+        <v>13.9</v>
+      </c>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>70.15000000000001</v>
+        <v>2.63</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0134</v>
+        <v>-0.0295</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>862740</v>
+        <v>28760000</v>
       </c>
       <c r="E599" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.7119</v>
       </c>
       <c r="F599" s="7" t="n">
-        <v>64.09</v>
+        <v>41.18</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="6" t="inlineStr"/>
+      <c r="I599" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
       <c r="J599" s="8" t="n">
-        <v>0.1431</v>
+        <v>-0.8093</v>
       </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26358,42 +26370,40 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>TCELL</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>115</v>
+        <v>148.6</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0566</v>
+        <v>-0.0237</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>21130000</v>
+        <v>1120000</v>
       </c>
       <c r="E600" s="4" t="n">
-        <v>0.4894</v>
+        <v>0.1071</v>
       </c>
       <c r="F600" s="3" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="G600" s="3" t="n">
-        <v>13.6</v>
-      </c>
+        <v>51.67</v>
+      </c>
+      <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="4" t="n">
-        <v>0.0735</v>
+        <v>-3.6635</v>
       </c>
       <c r="J600" s="4" t="n">
-        <v>0.1091</v>
+        <v>-0.4897</v>
       </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>İletişim</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST İLETİŞİM, BIST HİZMETLER, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26401,34 +26411,26 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>17.39</v>
+        <v>35.76</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.023</v>
+        <v>-0.0245</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>16640000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>5260000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>49.27</v>
-      </c>
-      <c r="G601" s="7" t="n">
-        <v>164.37</v>
-      </c>
+        <v>59.16</v>
+      </c>
+      <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
           <t>Üretici imalatı</t>
@@ -26436,7 +26438,7 @@
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26444,21 +26446,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>18.01</v>
+        <v>30.7</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0317</v>
+        <v>-0.0007000000000000001</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>61370000</v>
+        <v>26120000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>52.71</v>
+        <v>68.69</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26466,12 +26468,12 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26479,34 +26481,38 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>203.2</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0114</v>
+        <v>-0.0134</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>7230000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>862740</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>71.43000000000001</v>
+        <v>64.09</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="J603" s="8" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26514,21 +26520,23 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>205</v>
+        <v>244.25</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0029</v>
+        <v>-0.0338</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>11560000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>10010</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>53.72</v>
+        <v>45.91</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26536,55 +26544,45 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>35.16</v>
+        <v>6.06</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0228</v>
+        <v>-0.008199999999999999</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>5700000</v>
+        <v>44330000</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.8667</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>42.83</v>
-      </c>
-      <c r="G605" s="7" t="n">
-        <v>13.9</v>
-      </c>
+        <v>67.06999999999999</v>
+      </c>
+      <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26592,40 +26590,34 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>148.6</v>
+        <v>205</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0237</v>
+        <v>0.0029</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>1120000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>11560000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>51.67</v>
+        <v>53.72</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26633,67 +26625,75 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>80.04000000000001</v>
+        <v>6.34</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.009399999999999999</v>
+        <v>-0.0745</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>10710000</v>
-      </c>
-      <c r="E607" s="6" t="inlineStr"/>
+        <v>57090000</v>
+      </c>
+      <c r="E607" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F607" s="7" t="n">
-        <v>43.25</v>
+        <v>51.71</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="6" t="inlineStr"/>
-      <c r="J607" s="6" t="inlineStr"/>
-      <c r="K607" s="6" t="inlineStr"/>
-      <c r="L607" s="6" t="inlineStr"/>
+      <c r="I607" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J607" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
+      <c r="K607" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>19.78</v>
+        <v>203.2</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.0639</v>
+        <v>0.0114</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>711640</v>
-      </c>
-      <c r="E608" s="4" t="n">
-        <v>0.9869</v>
-      </c>
+        <v>7230000</v>
+      </c>
+      <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>60.87</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="4" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J608" s="4" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I608" s="2" t="inlineStr"/>
+      <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26701,34 +26701,42 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>2.88</v>
+        <v>17.39</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0368</v>
+        <v>-0.023</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>190570000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>16640000</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>52.36</v>
-      </c>
-      <c r="G609" s="6" t="inlineStr"/>
+        <v>49.27</v>
+      </c>
+      <c r="G609" s="7" t="n">
+        <v>164.37</v>
+      </c>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="I609" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J609" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26736,72 +26744,64 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>76.8</v>
+        <v>18.01</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0235</v>
+        <v>-0.0317</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>60180</v>
-      </c>
-      <c r="E610" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>61370000</v>
+      </c>
+      <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>43.15</v>
+        <v>52.71</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J610" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I610" s="2" t="inlineStr"/>
+      <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>9.6</v>
+        <v>6.12</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0194</v>
+        <v>-0.006500000000000001</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>961350</v>
-      </c>
-      <c r="E611" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>7340000</v>
+      </c>
+      <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>60.81</v>
+        <v>53.81</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J611" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I611" s="6" t="inlineStr"/>
+      <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr"/>
@@ -26829,7 +26829,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>12.05.2026 16:30</t>
+          <t>12.05.2026 17:31</t>
         </is>
       </c>
     </row>

</xml_diff>